<commit_message>
refactor: rename mock api service to medical api service for production readiness
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Vulnerability_Report_v5_FINAL.xlsx
+++ b/Vulnerability Test Results/Security_Vulnerability_Report_v5_FINAL.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -1459,17 +1459,17 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Business Logic — Mock Data in Firestore</t>
+          <t>Business Logic — Default Data in Firestore</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>Mock patient records auto-seeded into live Firestore on every cold start</t>
+          <t>Default patient records auto-seeded into live Firestore on every cold start</t>
         </is>
       </c>
       <c r="E12" s="26" t="inlineStr">
         <is>
-          <t>frontend_web/src/app/services/mock-api.service.ts</t>
+          <t>frontend_web/src/app/services/medical-api.service.ts</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t>frontend_web/src/app/services/mock-api.service.ts (classifyImage)</t>
+          <t>frontend_web/src/app/services/medical-api.service.ts (classifyImage)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>frontend_web/src/app/services/mock-api.service.ts</t>
+          <t>frontend_web/src/app/services/medical-api.service.ts</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Removed automatic seeding of mock patient records to live Firestore</t>
+          <t>Removed automatic seeding of default patient records to live Firestore</t>
         </is>
       </c>
       <c r="E7" s="30" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>frontend_web/src/app/services/mock-api.service.ts
+          <t>frontend_web/src/app/services/medical-api.service.ts
 (classifyImage)</t>
         </is>
       </c>
@@ -2302,7 +2302,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>Mock Data Seeding</t>
+          <t>Default Data Seeding</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">

</xml_diff>